<commit_message>
feat: excel_source valida fotos Canva del evento y fixture (tarea 16, SPEC 5.5)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/datos_ejemplo.xlsx
+++ b/tests/fixtures/datos_ejemplo.xlsx
@@ -786,7 +786,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX1</t>
+          <t>https://canva.link/fixfoto1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX2</t>
+          <t>https://canva.link/fixfoto2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX3</t>
+          <t>https://canva.link/fixfoto3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX4</t>
+          <t>https://canva.link/fixfoto4</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>

<commit_message>
feat: excel_source valida fotos Canva del evento y fixture (tarea 16, SPEC 5.5) (#2)
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/datos_ejemplo.xlsx
+++ b/tests/fixtures/datos_ejemplo.xlsx
@@ -786,7 +786,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX1</t>
+          <t>https://canva.link/fixfoto1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX2</t>
+          <t>https://canva.link/fixfoto2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX3</t>
+          <t>https://canva.link/fixfoto3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/uc?id=FIX4</t>
+          <t>https://canva.link/fixfoto4</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>

<commit_message>
feat: Event.fecha como date y parse_fecha (datetime o dd/mm/yyyy) (tarea 19, SPEC 5.4)
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/datos_ejemplo.xlsx
+++ b/tests/fixtures/datos_ejemplo.xlsx
@@ -19,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -678,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -820,6 +824,31 @@
         </is>
       </c>
       <c r="N2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46368</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Carrer de les Roselles, 32</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mercè Copado</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sergio Afonso</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>

</xml_diff>

<commit_message>
feat: Event.fecha como date y parse_fecha (datetime o dd/mm/yyyy) (tarea 19, SPEC 5.4) (#5)
Co-authored-by: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/datos_ejemplo.xlsx
+++ b/tests/fixtures/datos_ejemplo.xlsx
@@ -19,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -678,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -820,6 +824,31 @@
         </is>
       </c>
       <c r="N2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46368</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Carrer de les Roselles, 32</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mercè Copado</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sergio Afonso</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>

</xml_diff>